<commit_message>
Commit new pipeliend files
</commit_message>
<xml_diff>
--- a/Control Signals.xlsx
+++ b/Control Signals.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\Active HDL\Computer Architectuire\Pipleined_Processor_Design\Pipleined_Processor_Design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\GitHub\ENCS4370_Pipelined_32-bit_RISC_Processor_Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0FDE47F-CC63-42D4-906F-32738BAD1436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBE88473-3B06-4931-8573-6C88615A61A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DBFD7B10-F6DA-4103-8936-84779C32E9AC}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="61">
   <si>
     <t>OpCode</t>
   </si>
@@ -207,7 +207,7 @@
     <t>A4A3′​A2′</t>
   </si>
   <si>
-    <t>A4′A3′ + A4′A3A2′(A1 + A0′) + A4′A3A2(A1′ + A0) + A4A3′A2′A1A0</t>
+    <t>A4′​A3+A4A3′​A2′​</t>
   </si>
 </sst>
 </file>
@@ -1482,8 +1482,8 @@
       <c r="J12" s="4">
         <v>0</v>
       </c>
-      <c r="K12" s="4">
-        <v>1</v>
+      <c r="K12" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="L12" s="4">
         <v>1</v>
@@ -1553,8 +1553,8 @@
       <c r="J13" s="4">
         <v>0</v>
       </c>
-      <c r="K13" s="4">
-        <v>1</v>
+      <c r="K13" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="L13" s="4">
         <v>0</v>
@@ -1624,8 +1624,8 @@
       <c r="J14" s="4">
         <v>0</v>
       </c>
-      <c r="K14" s="4">
-        <v>1</v>
+      <c r="K14" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="L14" s="4">
         <v>0</v>
@@ -1695,8 +1695,8 @@
       <c r="J15" s="4">
         <v>0</v>
       </c>
-      <c r="K15" s="4">
-        <v>1</v>
+      <c r="K15" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="L15" s="4">
         <v>1</v>

</xml_diff>